<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-soundcard@cfda140f203ccbfb31539b21b99655dfad127fb0 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-soundcard-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-soundcard-bom.xlsx
@@ -277,7 +277,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="170">
   <si>
     <t>Row</t>
   </si>
@@ -414,9 +414,6 @@
     <t>LED_0805_2012Metric</t>
   </si>
   <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>1=K 2=A</t>
   </si>
   <si>
@@ -657,7 +654,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>9.0.7+1</t>
+    <t>10.0.1-10.0.1~ubuntu25.10.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -741,10 +738,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-04-21 20:40:12</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-04-22 16:06:20</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
   </si>
   <si>
     <t>Columns colors</t>
@@ -1638,7 +1635,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1651,13 +1648,13 @@
     </row>
     <row r="2" spans="1:11">
       <c r="C2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="3">
         <v>21</v>
@@ -1665,41 +1662,41 @@
     </row>
     <row r="3" spans="1:11">
       <c r="C3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="E3" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="C4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="E4" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="C5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>124</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -1707,13 +1704,13 @@
     </row>
     <row r="6" spans="1:11">
       <c r="C6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F6" s="3">
         <v>73</v>
@@ -1955,33 +1952,33 @@
         <v>18</v>
       </c>
       <c r="I14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="K14" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="45" customHeight="1">
       <c r="A15" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>50</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>21</v>
@@ -1990,10 +1987,10 @@
         <v>18</v>
       </c>
       <c r="I15" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>12</v>
@@ -2007,16 +2004,16 @@
         <v>12</v>
       </c>
       <c r="C16" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="E16" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>54</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>11</v>
@@ -2025,10 +2022,10 @@
         <v>18</v>
       </c>
       <c r="I16" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="J16" s="12" t="s">
         <v>56</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>57</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>12</v>
@@ -2042,28 +2039,28 @@
         <v>12</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>18</v>
       </c>
       <c r="I17" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>64</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>12</v>
@@ -2071,22 +2068,22 @@
     </row>
     <row r="18" spans="1:11" ht="30" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>66</v>
-      </c>
       <c r="F18" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G18" s="9" t="s">
         <v>17</v>
@@ -2095,10 +2092,10 @@
         <v>18</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>12</v>
@@ -2112,16 +2109,16 @@
         <v>12</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>69</v>
-      </c>
       <c r="F19" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>26</v>
@@ -2130,10 +2127,10 @@
         <v>18</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>12</v>
@@ -2141,22 +2138,22 @@
     </row>
     <row r="20" spans="1:11" ht="30" customHeight="1">
       <c r="A20" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="11" t="s">
+      <c r="E20" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>73</v>
-      </c>
       <c r="F20" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>35</v>
@@ -2165,10 +2162,10 @@
         <v>18</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>12</v>
@@ -2176,22 +2173,22 @@
     </row>
     <row r="21" spans="1:11" ht="30" customHeight="1">
       <c r="A21" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E21" s="7" t="s">
-        <v>77</v>
-      </c>
       <c r="F21" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>17</v>
@@ -2200,10 +2197,10 @@
         <v>18</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>12</v>
@@ -2211,22 +2208,22 @@
     </row>
     <row r="22" spans="1:11" ht="45" customHeight="1">
       <c r="A22" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="E22" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F22" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>82</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>11</v>
@@ -2235,10 +2232,10 @@
         <v>18</v>
       </c>
       <c r="I22" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="J22" s="12" t="s">
         <v>83</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>84</v>
       </c>
       <c r="K22" s="10" t="s">
         <v>12</v>
@@ -2246,22 +2243,22 @@
     </row>
     <row r="23" spans="1:11" ht="30" customHeight="1">
       <c r="A23" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E23" s="7" t="s">
-        <v>88</v>
-      </c>
       <c r="F23" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>26</v>
@@ -2270,10 +2267,10 @@
         <v>18</v>
       </c>
       <c r="I23" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="J23" s="8" t="s">
         <v>89</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>90</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>12</v>
@@ -2281,22 +2278,22 @@
     </row>
     <row r="24" spans="1:11" ht="30" customHeight="1">
       <c r="A24" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="11" t="s">
+      <c r="D24" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="F24" s="11" t="s">
         <v>94</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>95</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>11</v>
@@ -2305,10 +2302,10 @@
         <v>18</v>
       </c>
       <c r="I24" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="J24" s="12" t="s">
         <v>96</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>97</v>
       </c>
       <c r="K24" s="10" t="s">
         <v>12</v>
@@ -2316,22 +2313,22 @@
     </row>
     <row r="25" spans="1:11" ht="30" customHeight="1">
       <c r="A25" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>11</v>
@@ -2340,10 +2337,10 @@
         <v>18</v>
       </c>
       <c r="I25" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>12</v>
@@ -2351,22 +2348,22 @@
     </row>
     <row r="26" spans="1:11" ht="30" customHeight="1">
       <c r="A26" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="11" t="s">
+      <c r="D26" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="E26" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="F26" s="11" t="s">
         <v>108</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>109</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>11</v>
@@ -2375,10 +2372,10 @@
         <v>18</v>
       </c>
       <c r="I26" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="J26" s="12" t="s">
         <v>110</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>111</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>12</v>
@@ -2386,22 +2383,22 @@
     </row>
     <row r="27" spans="1:11" ht="30" customHeight="1">
       <c r="A27" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>114</v>
-      </c>
       <c r="F27" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>11</v>
@@ -2410,10 +2407,10 @@
         <v>18</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>12</v>
@@ -2437,7 +2434,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="40.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
@@ -2448,7 +2445,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2461,13 +2458,13 @@
     </row>
     <row r="2" spans="1:11">
       <c r="C2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" s="3">
         <v>21</v>
@@ -2475,41 +2472,41 @@
     </row>
     <row r="3" spans="1:11">
       <c r="C3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="E3" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="C4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="E4" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="C5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>124</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -2517,13 +2514,13 @@
     </row>
     <row r="6" spans="1:11">
       <c r="C6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F6" s="3">
         <v>73</v>
@@ -2572,28 +2569,28 @@
         <v>12</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>137</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H9" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I9" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>12</v>
@@ -2607,28 +2604,28 @@
         <v>12</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>11</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>12</v>
@@ -2661,7 +2658,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -2670,13 +2667,13 @@
     </row>
     <row r="2" spans="1:8">
       <c r="D2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="G2" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -2684,13 +2681,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="D3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="G3" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -2699,13 +2696,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="D4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="G4" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H28)</f>
@@ -2714,23 +2711,23 @@
     </row>
     <row r="5" spans="1:8">
       <c r="D5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -2754,16 +2751,16 @@
         <v>5</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="18" t="s">
         <v>145</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1">
@@ -2796,7 +2793,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>16</v>
@@ -2887,7 +2884,7 @@
         <v>43</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D15" s="19" t="s">
         <v>44</v>
@@ -2903,16 +2900,16 @@
     </row>
     <row r="16" spans="1:8" ht="45" customHeight="1">
       <c r="A16" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="E16" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>51</v>
       </c>
       <c r="F16" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -2925,16 +2922,16 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" s="19" t="s">
+      <c r="E17" s="19" t="s">
         <v>55</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>56</v>
       </c>
       <c r="F17" s="19">
         <f>BoardQty*1</f>
@@ -2947,16 +2944,16 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="D18" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="19" t="s">
-        <v>61</v>
-      </c>
       <c r="E18" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F18" s="19">
         <f>CEILING(BoardQty*10,1)</f>
@@ -2969,16 +2966,16 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="19" t="s">
-        <v>66</v>
-      </c>
       <c r="D19" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F19" s="19">
         <f>CEILING(BoardQty*4,1)</f>
@@ -2991,16 +2988,16 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B20" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="19" t="s">
-        <v>69</v>
-      </c>
       <c r="D20" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F20" s="19">
         <f>CEILING(BoardQty*3,1)</f>
@@ -3013,16 +3010,16 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>73</v>
-      </c>
       <c r="D21" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F21" s="19">
         <f>CEILING(BoardQty*5,1)</f>
@@ -3035,16 +3032,16 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>77</v>
-      </c>
       <c r="D22" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F22" s="19">
         <f>CEILING(BoardQty*4,1)</f>
@@ -3057,16 +3054,16 @@
     </row>
     <row r="23" spans="1:8" ht="45" customHeight="1">
       <c r="A23" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B23" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="19" t="s">
+      <c r="E23" s="19" t="s">
         <v>82</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>83</v>
       </c>
       <c r="F23" s="19">
         <f>BoardQty*1</f>
@@ -3079,19 +3076,19 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="C24" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="E24" s="19" t="s">
         <v>88</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>89</v>
       </c>
       <c r="F24" s="19">
         <f>CEILING(BoardQty*3,1)</f>
@@ -3104,16 +3101,16 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="E25" s="19" t="s">
         <v>95</v>
-      </c>
-      <c r="E25" s="19" t="s">
-        <v>96</v>
       </c>
       <c r="F25" s="19">
         <f>BoardQty*1</f>
@@ -3126,16 +3123,16 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="D26" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="E26" s="19" t="s">
         <v>102</v>
-      </c>
-      <c r="E26" s="19" t="s">
-        <v>103</v>
       </c>
       <c r="F26" s="19">
         <f>BoardQty*1</f>
@@ -3148,16 +3145,16 @@
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1">
       <c r="A27" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="D27" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="E27" s="19" t="s">
         <v>109</v>
-      </c>
-      <c r="E27" s="19" t="s">
-        <v>110</v>
       </c>
       <c r="F27" s="19">
         <f>BoardQty*1</f>
@@ -3170,16 +3167,16 @@
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
       <c r="A28" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B28" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="B28" s="19" t="s">
-        <v>114</v>
-      </c>
       <c r="D28" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="19" t="s">
         <v>109</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>110</v>
       </c>
       <c r="F28" s="19">
         <f>BoardQty*1</f>
@@ -3192,15 +3189,15 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B31" s="22" t="s">
         <v>153</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="23" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3338,14 +3335,14 @@
     <col min="2" max="2" width="11.7109375" customWidth="1"/>
     <col min="3" max="3" width="36.7109375" customWidth="1" outlineLevel="2"/>
     <col min="4" max="4" width="59.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="21.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="28.7109375" customWidth="1" outlineLevel="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
     <col min="7" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -3353,13 +3350,13 @@
     </row>
     <row r="2" spans="1:7">
       <c r="D2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="F2" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G2" s="13">
         <v>1</v>
@@ -3367,13 +3364,13 @@
     </row>
     <row r="3" spans="1:7">
       <c r="D3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>120</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -3382,13 +3379,13 @@
     </row>
     <row r="4" spans="1:7">
       <c r="D4" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="F4" s="14" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G4" s="16">
         <f>SUM(G10:G11)</f>
@@ -3397,23 +3394,23 @@
     </row>
     <row r="5" spans="1:7">
       <c r="D5" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="D6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -3433,30 +3430,30 @@
         <v>5</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="E9" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="F9" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>145</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="C10" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="C10" s="19" t="s">
-        <v>137</v>
-      </c>
       <c r="D10" s="19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E10" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -3469,16 +3466,16 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="19" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E11" s="19">
         <f>BoardQty*1</f>
@@ -3491,15 +3488,15 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="22" t="s">
         <v>153</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="23" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3537,77 +3534,77 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="25" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="26" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="29" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="30" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="31" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-soundcard@dc562330052bb9dca7300b94083724d9ba66bf31 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-soundcard-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-soundcard-bom.xlsx
@@ -738,10 +738,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-05-12 07:03:03</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
+    <t>2026-05-13 11:22:37</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.9.0</t>
   </si>
   <si>
     <t>Columns colors</t>

</xml_diff>